<commit_message>
Solve bug in asignacion_tianguis.model.js
</commit_message>
<xml_diff>
--- a/back/src/templates/reporte_total_generales_template.xlsx
+++ b/back/src/templates/reporte_total_generales_template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\DEV\tianguis\back\src\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4E6B8ABA-5D8B-4D37-A01D-11FF8512EE64}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5E871987-5838-4AC0-8162-E112B9B89C85}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -98,16 +98,16 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>352425</xdr:colOff>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>342900</xdr:colOff>
       <xdr:row>0</xdr:row>
-      <xdr:rowOff>123825</xdr:rowOff>
+      <xdr:rowOff>152400</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>19880</xdr:colOff>
-      <xdr:row>2</xdr:row>
-      <xdr:rowOff>219075</xdr:rowOff>
+      <xdr:colOff>1820105</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>9525</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -130,7 +130,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="1143000" y="123825"/>
+          <a:off x="1485900" y="152400"/>
           <a:ext cx="1477205" cy="476250"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -409,18 +409,18 @@
   <dimension ref="F3"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="11.85546875" customWidth="1"/>
-    <col min="2" max="2" width="27.140625" customWidth="1"/>
-    <col min="3" max="3" width="14.140625" customWidth="1"/>
-    <col min="4" max="4" width="14.5703125" customWidth="1"/>
+    <col min="1" max="1" width="11.28515625" customWidth="1"/>
+    <col min="2" max="2" width="5.85546875" customWidth="1"/>
+    <col min="3" max="3" width="31.7109375" customWidth="1"/>
+    <col min="4" max="4" width="16.5703125" customWidth="1"/>
     <col min="5" max="5" width="15.85546875" customWidth="1"/>
-    <col min="6" max="6" width="15.140625" customWidth="1"/>
-    <col min="7" max="7" width="14" customWidth="1"/>
-    <col min="8" max="8" width="13.28515625" customWidth="1"/>
-    <col min="9" max="9" width="13.7109375" customWidth="1"/>
-    <col min="10" max="10" width="13.85546875" customWidth="1"/>
-    <col min="11" max="11" width="17.7109375" customWidth="1"/>
-    <col min="12" max="12" width="16.140625" customWidth="1"/>
+    <col min="6" max="7" width="15.140625" customWidth="1"/>
+    <col min="8" max="8" width="14.5703125" customWidth="1"/>
+    <col min="9" max="9" width="16" customWidth="1"/>
+    <col min="10" max="10" width="15" customWidth="1"/>
+    <col min="11" max="11" width="14" customWidth="1"/>
+    <col min="12" max="12" width="17.7109375" customWidth="1"/>
+    <col min="13" max="13" width="17.140625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="3" spans="6:6" ht="18.75" x14ac:dyDescent="0.3">

</xml_diff>